<commit_message>
docs: final update to help and user documentation
</commit_message>
<xml_diff>
--- a/docs/Bug_Ledger.xlsx
+++ b/docs/Bug_Ledger.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="506" documentId="8_{11E06D47-9345-41BE-A197-12778AEAB68C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0AD5875-4499-45A8-BEA9-901E0AD8DC72}"/>
   <bookViews>
-    <workbookView xWindow="8196" yWindow="240" windowWidth="14844" windowHeight="12156" xr2:uid="{705CAC83-FD9A-4432-901E-BE6C90701170}"/>
+    <workbookView xWindow="9408" yWindow="84" windowWidth="12792" windowHeight="12156" xr2:uid="{705CAC83-FD9A-4432-901E-BE6C90701170}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1644,9 +1644,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1656,9 +1653,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1666,6 +1660,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1683,19 +1683,6 @@
         <vertAlign val="baseline"/>
         <sz val="14"/>
         <color theme="1"/>
-        <family val="2"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1794,6 +1781,19 @@
         <vertAlign val="baseline"/>
         <sz val="14"/>
         <color theme="1"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <family val="2"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1839,20 +1839,24 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{17BDC1F7-5D53-4DCD-9908-F2256780EA89}" name="Table2" displayName="Table2" ref="B7:K34" totalsRowShown="0" headerRowDxfId="11" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{17BDC1F7-5D53-4DCD-9908-F2256780EA89}" name="Table2" displayName="Table2" ref="B7:K34" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="B7:K34" xr:uid="{17BDC1F7-5D53-4DCD-9908-F2256780EA89}"/>
   <tableColumns count="10">
-    <tableColumn id="10" xr3:uid="{1D6962DF-84E7-4EF0-9D0B-698844FE025F}" name="PHASES:" dataDxfId="10"/>
-    <tableColumn id="1" xr3:uid="{6B63600E-CBD0-42CB-88AB-E2ACAE9EAF0B}" name="ISSUE:" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{6D130CB6-6F52-4C75-9D37-1D063CCE2542}" name="Date:" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{202EB460-4F10-4EAB-9D7F-C833B3FD20E5}" name="Reported:" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{1A0BFD4B-74B4-46F9-B51F-2C54F6282908}" name="Assigned:" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{24DF0A62-7A90-403B-A02F-6A7E001A7407}" name="Priority: (Low, Med, High, Critical)" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{3DEEEF1A-6C1B-40F0-A25C-0B5F668BE6A9}" name="Status: (Open, In progress, Resolved)" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{38109E21-DF40-4CC7-A2C6-2872F559927B}" name="Resolution: _x000a_[Explanation of how the issue was resolved, including any code changes or fixes applied.]" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{D495AA50-6BE3-4F07-914F-6D577C6CB85A}" name="Attachments: _x000a_[Links or references to any relevant files, screenshots, or documents related to the issue.]" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{899E85F6-A5E6-4B08-AFA5-DC5D7ED87965}" name="Comments (if any):" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{1D6962DF-84E7-4EF0-9D0B-698844FE025F}" name="PHASES:" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{6B63600E-CBD0-42CB-88AB-E2ACAE9EAF0B}" name="ISSUE:" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{6D130CB6-6F52-4C75-9D37-1D063CCE2542}" name="Date:" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{202EB460-4F10-4EAB-9D7F-C833B3FD20E5}" name="Reported:" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{1A0BFD4B-74B4-46F9-B51F-2C54F6282908}" name="Assigned:" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{24DF0A62-7A90-403B-A02F-6A7E001A7407}" name="Priority: (Low, Med, High, Critical)" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{3DEEEF1A-6C1B-40F0-A25C-0B5F668BE6A9}" name="Status: (Open, In progress, Resolved)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{38109E21-DF40-4CC7-A2C6-2872F559927B}" name="Resolution: _x000a_[Explanation of how the issue was resolved, including any code changes or fixes applied.]" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{D495AA50-6BE3-4F07-914F-6D577C6CB85A}" name="Attachments: _x000a_[Links or references to any relevant files, screenshots, or documents related to the issue.]" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{899E85F6-A5E6-4B08-AFA5-DC5D7ED87965}" name="Comments (if any):" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2192,34 +2196,34 @@
     <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:12" s="10" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" s="9" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="8"/>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:12" s="14" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="13" t="s">
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+    </row>
+    <row r="5" spans="1:12" s="12" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
@@ -2260,751 +2264,751 @@
       <c r="L7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="180.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="13">
         <v>46100</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="13">
         <v>46100</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="K8" s="11" t="s">
+      <c r="K8" s="10" t="s">
         <v>92</v>
       </c>
       <c r="L8" s="2"/>
     </row>
     <row r="9" spans="1:12" ht="222.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="11"/>
-      <c r="C9" s="11" t="s">
+      <c r="B9" s="10"/>
+      <c r="C9" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="13">
         <v>46100</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="13">
         <v>46100</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I9" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="J9" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="K9" s="11" t="s">
+      <c r="K9" s="10" t="s">
         <v>87</v>
       </c>
       <c r="L9" s="2"/>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="11"/>
-      <c r="C10" s="16" t="s">
+      <c r="B10" s="10"/>
+      <c r="C10" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="13">
         <v>46096</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="13">
         <v>46096</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="J10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="K10" s="10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="11"/>
-      <c r="C11" s="11" t="s">
+      <c r="B11" s="10"/>
+      <c r="C11" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="13">
         <v>46096</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="13">
         <v>46096</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="H11" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="I11" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J11" s="11" t="s">
+      <c r="J11" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="K11" s="11"/>
+      <c r="K11" s="10"/>
       <c r="L11" s="2"/>
     </row>
     <row r="12" spans="1:12" ht="70.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="11"/>
-      <c r="C12" s="11" t="s">
+      <c r="B12" s="10"/>
+      <c r="C12" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="13">
         <v>46097</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="13">
         <v>46097</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="11" t="s">
+      <c r="I12" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="J12" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="11"/>
+      <c r="K12" s="10"/>
       <c r="L12" s="2"/>
     </row>
     <row r="13" spans="1:12" s="2" customFormat="1" ht="70.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="11"/>
-      <c r="C13" s="11" t="s">
+      <c r="B13" s="10"/>
+      <c r="C13" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="13">
         <v>46097</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="13">
         <v>46097</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="I13" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="11"/>
+      <c r="K13" s="10"/>
     </row>
     <row r="14" spans="1:12" s="2" customFormat="1" ht="70.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="11"/>
-      <c r="C14" s="11" t="s">
+      <c r="B14" s="10"/>
+      <c r="C14" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="13">
         <v>46098</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="13">
         <v>46098</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I14" s="11" t="s">
+      <c r="I14" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
     </row>
     <row r="15" spans="1:12" s="2" customFormat="1" ht="82.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="13">
         <v>46099</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="13">
         <v>46099</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="I15" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="K15" s="11"/>
+      <c r="K15" s="10"/>
     </row>
     <row r="16" spans="1:12" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="11"/>
-      <c r="C16" s="11" t="s">
+      <c r="B16" s="10"/>
+      <c r="C16" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="13">
         <v>46099</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="13">
         <v>46099</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="I16" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
       <c r="L16" s="2"/>
     </row>
     <row r="17" spans="2:12" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="11"/>
-      <c r="C17" s="11" t="s">
+      <c r="B17" s="10"/>
+      <c r="C17" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="13">
         <v>46100</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="13">
         <v>46100</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="H17" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I17" s="11" t="s">
+      <c r="I17" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
       <c r="L17" s="2"/>
     </row>
     <row r="18" spans="2:12" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="11"/>
-      <c r="C18" s="11" t="s">
+      <c r="B18" s="10"/>
+      <c r="C18" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="13">
         <v>46100</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="13">
         <v>46100</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I18" s="11" t="s">
+      <c r="I18" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
       <c r="L18" s="2"/>
     </row>
     <row r="19" spans="2:12" ht="120" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="11"/>
-      <c r="C19" s="11" t="s">
+      <c r="B19" s="10"/>
+      <c r="C19" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="13">
         <v>46101</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="13">
         <v>46101</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="H19" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I19" s="11" t="s">
+      <c r="I19" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
       <c r="L19" s="2"/>
     </row>
     <row r="20" spans="2:12" ht="111" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="13">
         <v>46104</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="13">
         <v>46104</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="H20" s="11" t="s">
+      <c r="H20" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I20" s="11" t="s">
+      <c r="I20" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
       <c r="L20" s="2"/>
     </row>
     <row r="21" spans="2:12" s="2" customFormat="1" ht="112.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="11"/>
-      <c r="C21" s="11" t="s">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="13">
         <v>46104</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="13">
         <v>46104</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="H21" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I21" s="11" t="s">
+      <c r="I21" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
     </row>
     <row r="22" spans="2:12" s="2" customFormat="1" ht="122.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="11"/>
-      <c r="C22" s="11" t="s">
+      <c r="B22" s="10"/>
+      <c r="C22" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="13">
         <v>46104</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="13">
         <v>46104</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="H22" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I22" s="11" t="s">
+      <c r="I22" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
     </row>
     <row r="23" spans="2:12" s="2" customFormat="1" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="11"/>
-      <c r="C23" s="11" t="s">
+      <c r="B23" s="10"/>
+      <c r="C23" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="13">
         <v>46084</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="13">
         <v>46104</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="G23" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="11" t="s">
+      <c r="H23" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I23" s="11" t="s">
+      <c r="I23" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
     </row>
     <row r="24" spans="2:12" s="2" customFormat="1" ht="111" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="11"/>
-      <c r="C24" s="11" t="s">
+      <c r="B24" s="10"/>
+      <c r="C24" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="13">
         <v>46104</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="13">
         <v>46104</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="H24" s="11" t="s">
+      <c r="H24" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I24" s="11" t="s">
+      <c r="I24" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
     </row>
     <row r="25" spans="2:12" s="2" customFormat="1" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="13">
         <v>46102</v>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="13">
         <v>46102</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F25" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="G25" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H25" s="11" t="s">
+      <c r="H25" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I25" s="11" t="s">
+      <c r="I25" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
     </row>
     <row r="26" spans="2:12" s="2" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="11"/>
-      <c r="C26" s="11" t="s">
+      <c r="B26" s="10"/>
+      <c r="C26" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="13">
         <v>46102</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="13">
         <v>46102</v>
       </c>
-      <c r="F26" s="11" t="s">
+      <c r="F26" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H26" s="11" t="s">
+      <c r="H26" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I26" s="11" t="s">
+      <c r="I26" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="J26" s="11"/>
-      <c r="K26" s="11"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
     </row>
     <row r="27" spans="2:12" s="2" customFormat="1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="11"/>
-      <c r="C27" s="11" t="s">
+      <c r="B27" s="10"/>
+      <c r="C27" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="13">
         <v>46103</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="13">
         <v>46103</v>
       </c>
-      <c r="F27" s="11" t="s">
+      <c r="F27" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G27" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="11" t="s">
+      <c r="H27" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I27" s="11" t="s">
+      <c r="I27" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
     </row>
     <row r="28" spans="2:12" s="2" customFormat="1" ht="132.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="11"/>
-      <c r="C28" s="16" t="s">
+      <c r="B28" s="10"/>
+      <c r="C28" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="13">
         <v>46104</v>
       </c>
-      <c r="E28" s="15">
+      <c r="E28" s="13">
         <v>46104</v>
       </c>
-      <c r="F28" s="11" t="s">
+      <c r="F28" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G28" s="11" t="s">
+      <c r="G28" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H28" s="11" t="s">
+      <c r="H28" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I28" s="11" t="s">
+      <c r="I28" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
     </row>
     <row r="29" spans="2:12" s="2" customFormat="1" ht="114.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="11"/>
-      <c r="C29" s="11" t="s">
+      <c r="B29" s="10"/>
+      <c r="C29" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="13">
         <v>46104</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="13">
         <v>46104</v>
       </c>
-      <c r="F29" s="11" t="s">
+      <c r="F29" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="G29" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H29" s="11" t="s">
+      <c r="H29" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I29" s="11" t="s">
+      <c r="I29" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
     </row>
     <row r="30" spans="2:12" s="2" customFormat="1" ht="187.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="13">
         <v>46104</v>
       </c>
-      <c r="E30" s="15">
+      <c r="E30" s="13">
         <v>46104</v>
       </c>
-      <c r="F30" s="11" t="s">
+      <c r="F30" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="G30" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="H30" s="11" t="s">
+      <c r="H30" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I30" s="11" t="s">
+      <c r="I30" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="J30" s="11"/>
-      <c r="K30" s="11" t="s">
+      <c r="J30" s="10"/>
+      <c r="K30" s="10" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="31" spans="2:12" s="2" customFormat="1" ht="216" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="11"/>
-      <c r="C31" s="11" t="s">
+      <c r="B31" s="10"/>
+      <c r="C31" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="13">
         <v>46104</v>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="13">
         <v>46104</v>
       </c>
-      <c r="F31" s="11" t="s">
+      <c r="F31" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G31" s="11" t="s">
+      <c r="G31" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="H31" s="11" t="s">
+      <c r="H31" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I31" s="11" t="s">
+      <c r="I31" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="J31" s="11"/>
-      <c r="K31" s="11" t="s">
+      <c r="J31" s="10"/>
+      <c r="K31" s="10" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="32" spans="2:12" s="2" customFormat="1" ht="184.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="11"/>
-      <c r="C32" s="11" t="s">
+      <c r="B32" s="10"/>
+      <c r="C32" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="13">
         <v>46103</v>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="13">
         <v>46103</v>
       </c>
-      <c r="F32" s="11" t="s">
+      <c r="F32" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G32" s="11" t="s">
+      <c r="G32" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H32" s="11" t="s">
+      <c r="H32" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I32" s="11" t="s">
+      <c r="I32" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
     </row>
     <row r="33" spans="2:12" s="2" customFormat="1" ht="165" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="11"/>
-      <c r="C33" s="11" t="s">
+      <c r="B33" s="10"/>
+      <c r="C33" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="13">
         <v>46104</v>
       </c>
-      <c r="E33" s="15">
+      <c r="E33" s="13">
         <v>46104</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="F33" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G33" s="11" t="s">
+      <c r="G33" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H33" s="11" t="s">
+      <c r="H33" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I33" s="11" t="s">
+      <c r="I33" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="J33" s="16" t="s">
+      <c r="J33" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="K33" s="11"/>
+      <c r="K33" s="10"/>
     </row>
     <row r="34" spans="2:12" s="2" customFormat="1" ht="205.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="11"/>
-      <c r="C34" s="11" t="s">
+      <c r="B34" s="10"/>
+      <c r="C34" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D34" s="15">
+      <c r="D34" s="13">
         <v>46104</v>
       </c>
-      <c r="E34" s="15">
+      <c r="E34" s="13">
         <v>46104</v>
       </c>
-      <c r="F34" s="11" t="s">
+      <c r="F34" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G34" s="11" t="s">
+      <c r="G34" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="H34" s="11" t="s">
+      <c r="H34" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I34" s="11" t="s">
+      <c r="I34" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="J34" s="11"/>
-      <c r="K34" s="11" t="s">
+      <c r="J34" s="10"/>
+      <c r="K34" s="10" t="s">
         <v>54</v>
       </c>
     </row>

</xml_diff>